<commit_message>
[rp_BangluongP(GopDC).rpt,rp_BangluongP(GopYS).rpt,rp_BangluongP.rpt] > Sua cac report bang luong bi che mat so tien do font qua lon
</commit_message>
<xml_diff>
--- a/DinhKy/BPM/ThongKeBPM统计表.xlsx
+++ b/DinhKy/BPM/ThongKeBPM统计表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/743d27c10fd000ba/YIHSHUO/GIT/Yihshuo_Script/DinhKy/BPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{7BEFC58D-BABB-482A-97B7-6BFB1ACAA2BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E224BCB-90EB-475B-9437-0BE9513BA2D4}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{7BEFC58D-BABB-482A-97B7-6BFB1ACAA2BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{777C90F2-88F9-4263-89D6-68F7A3771B11}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="215">
   <si>
     <t>ĐƠN ĐỀ NGHỊ ĐI CÔNG TÁC</t>
   </si>
@@ -607,15 +607,9 @@
     <t>DANH SÁCH XÉT KÝ HĐLĐ SAU 06 NGÀY</t>
   </si>
   <si>
-    <t>DANH SÁCH NHÀ CUNG ỨNG ĐẠT YÊU CẦU</t>
-  </si>
-  <si>
     <t>BẢNG THỐNG KÊ CHẤT LƯỢNG VÀ NGÀY GIAO HÀNG CỦA NHÀ CUNG ỨNG</t>
   </si>
   <si>
-    <t>BẢNG TỔNG KẾT ĐÁNH GIÁ ĐỊNH KỲ NHÀ CUNG ỨNG</t>
-  </si>
-  <si>
     <t>BẢNG CHỈNH SỬA THÔNG TIN NHÀ CUNG ỨNG</t>
   </si>
   <si>
@@ -632,9 +626,6 @@
   </si>
   <si>
     <t>Thông báo tái chế</t>
-  </si>
-  <si>
-    <t>Phiếu bù</t>
   </si>
   <si>
     <t>Phiếu xuất vật tư (ERP)</t>
@@ -721,6 +712,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>（设计</t>
     </r>
@@ -738,6 +731,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>）</t>
     </r>
@@ -771,6 +766,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>加上一栏计算单位</t>
     </r>
@@ -788,6 +785,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>抽检数量</t>
     </r>
@@ -805,6 +804,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>不良双数</t>
     </r>
@@ -822,6 +823,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>在</t>
     </r>
@@ -839,6 +842,8 @@
         <sz val="11"/>
         <color rgb="FFC00000"/>
         <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>→</t>
     </r>
@@ -1874,143 +1879,801 @@
     <t>Nhân sự đòi hỏi Người lao động phải ký tên trên đơn.</t>
   </si>
   <si>
-    <t>v</t>
+    <t>Đơn vị chưa thống nhất được lưu trình</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>供應商品質與交期統計表</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>PHIẾU ĐỀ NGHỊ LOẠI BỎ NHÀ CUNG ỨNG</t>
+  </si>
+  <si>
+    <t>刪除不合格供應商建議表</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BẢNG TƯ LIỆU NHÀ CUNG ỨNG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>供應商資料表</t>
+    </r>
+  </si>
+  <si>
+    <t>Đã Công Bố 已发布</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BẢNG CHỈNH SỬA THÔNG TIN NHÀ CUNG ỨNG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>修改供應商資料表</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BẢNG THỐNG KÊ CHẤT LƯỢNG VÀ NGÀY GIAO HÀNG CỦA NHÀ CUNG ỨNG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>供應商品質與交期統計表</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BẢNG TỔNG KẾT ĐÁNH GIÁ ĐỊNH KỲ NHÀ CUNG ỨNG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>供應商定期評鑑彙總表</t>
+    </r>
+  </si>
+  <si>
+    <t>Chưa có lưu trình 尚未有流程</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU THÔNG BÁO ĐỐI SÁCH CẢI TIẾN NHÀ CUNG ỨNG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>供應商改善對策通知單</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>PHIẾU ĐỀ NGHỊ LOẠI BỎ NHÀ CUNG ỨNG</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>刪除不合格供應商建議表</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ĐƠN XIN ĐẶT MUA HÀNG </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>請</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>購</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  
+A-TM-QP009-07C</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU ĐẶT MUA HÀNG </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>採</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>購</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+A-TM-QP009-08C (ERP)                   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>　</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">             </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU ĐẶT MUA HÀNG </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>採</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>購</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+A-TM-QP009-09B (ERP)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU ĐẶT MUA HÀNG ( TSCĐ)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>採購單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>固定資產</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU NHẬP KHO </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>入庫單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+A-TM-QP009-14B (ERP)            </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU NGHIỆM THU TSCĐ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>固定資產驗收單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+T-DCC-002B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU NHẬP TÀI SẢN CỐ ĐỊNH 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>固</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>定</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>財</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>產</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>入</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>庫</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+T-TV-027B(ERP)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU CHUYỂN GIAO (TRẢ) HÀNG </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>交</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>退</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>料</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">    A-KVT-QP018-04B             </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU THANH TOÁN NGOẠI TỆ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>外匯請款單</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 
+T-DCC-014B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PHIẾU THANH TOÁN </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>請</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>款</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="DFKai-SB"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單</t>
+    </r>
+  </si>
+  <si>
+    <t>Các mẫu của Tỷ Xuân</t>
+  </si>
+  <si>
+    <t>采购</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>Đơ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>n v</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>ị</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ch</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>ư</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>a th</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>ố</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ng nh</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>ấ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">t </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>đượ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>c l</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Cambria"/>
-        <family val="1"/>
-      </rPr>
-      <t>ư</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>u trình</t>
-    </r>
+    <t>正在设计</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>主管不接受</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -2018,7 +2681,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="32">
+  <fonts count="35">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2148,6 +2811,8 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2231,22 +2896,48 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="1"/>
+      <color rgb="FF081B3A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="DengXian"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="DFKai-SB"/>
+      <family val="4"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="DFKai-SB"/>
+      <family val="4"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2264,7 +2955,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2394,7 +3085,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2430,12 +3121,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2452,9 +3137,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2498,15 +3180,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2516,6 +3223,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2534,8 +3244,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2546,11 +3259,23 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2959,12 +3684,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="19"/>
+    <col min="1" max="1" width="9.125" style="17"/>
     <col min="2" max="2" width="55.75" style="3" customWidth="1"/>
-    <col min="3" max="3" width="39.25" style="3" customWidth="1"/>
+    <col min="3" max="3" width="41.125" style="3" customWidth="1"/>
     <col min="4" max="4" width="27.25" style="3" customWidth="1"/>
     <col min="5" max="5" width="19" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.625" style="3" bestFit="1" customWidth="1"/>
@@ -2976,49 +3701,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="59.25" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
     </row>
     <row r="2" spans="1:10" ht="37.5" customHeight="1">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="52" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="55" t="s">
         <v>61</v>
       </c>
       <c r="C2" s="49"/>
       <c r="D2" s="5"/>
-      <c r="E2" s="45" t="s">
+      <c r="E2" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="45" t="s">
+      <c r="F2" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="45" t="s">
+      <c r="G2" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="H2" s="45" t="s">
-        <v>175</v>
-      </c>
-      <c r="I2" s="45" t="s">
-        <v>176</v>
-      </c>
-      <c r="J2" s="45" t="s">
+      <c r="H2" s="52" t="s">
+        <v>172</v>
+      </c>
+      <c r="I2" s="52" t="s">
+        <v>173</v>
+      </c>
+      <c r="J2" s="52" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="28.5">
-      <c r="A3" s="46"/>
+      <c r="A3" s="53"/>
       <c r="B3" s="6" t="s">
         <v>66</v>
       </c>
@@ -3028,12 +3753,12 @@
       <c r="D3" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="7">
@@ -3821,10 +4546,10 @@
         <v>122</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>36</v>
@@ -3835,20 +4560,20 @@
       <c r="I38" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J38" s="36"/>
+      <c r="J38" s="33"/>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="7">
         <v>36</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>37</v>
@@ -3859,7 +4584,7 @@
       <c r="I39" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J39" s="36"/>
+      <c r="J39" s="33"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="7">
@@ -3872,7 +4597,7 @@
         <v>107</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E40" s="9" t="s">
         <v>37</v>
@@ -3890,16 +4615,16 @@
         <v>38</v>
       </c>
       <c r="B41" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="E41" s="7" t="s">
         <v>178</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="F41" s="7"/>
       <c r="G41" s="11"/>
@@ -3907,23 +4632,23 @@
       <c r="I41" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J41" s="36"/>
+      <c r="J41" s="33"/>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="7">
         <v>39</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="F42" s="7"/>
       <c r="G42" s="11"/>
@@ -3931,111 +4656,113 @@
       <c r="I42" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J42" s="36"/>
+      <c r="J42" s="33"/>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1">
       <c r="A43" s="7">
         <v>40</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E43" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="C43" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="D43" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="E43" s="13" t="s">
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I43" s="7"/>
+      <c r="J43" s="56" t="s">
         <v>187</v>
-      </c>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="I43" s="13"/>
-      <c r="J43" s="53" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="15" customHeight="1">
       <c r="A44" s="7">
         <v>41</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="C44" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D44" s="12"/>
-      <c r="E44" s="13" t="s">
+      <c r="D44" s="8"/>
+      <c r="E44" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13" t="s">
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="I44" s="13"/>
-      <c r="J44" s="54"/>
-    </row>
-    <row r="45" spans="1:10" ht="14.25" customHeight="1">
+      <c r="I44" s="7"/>
+      <c r="J44" s="57"/>
+    </row>
+    <row r="45" spans="1:10">
       <c r="A45" s="7">
         <v>42</v>
       </c>
-      <c r="B45" s="37" t="s">
+      <c r="B45" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D45" s="12" t="s">
+      <c r="D45" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="I45" s="14"/>
+      <c r="J45" s="36" t="s">
         <v>188</v>
       </c>
-      <c r="E45" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
-      <c r="H45" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="I45" s="38"/>
-      <c r="J45" s="54"/>
     </row>
     <row r="46" spans="1:10" ht="28.5">
       <c r="A46" s="7">
         <v>43</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="E46" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="14" t="s">
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="I46" s="38"/>
-      <c r="J46" s="39" t="s">
-        <v>189</v>
+      <c r="I46" s="14"/>
+      <c r="J46" s="34" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="7">
         <v>44</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="13" t="s">
         <v>111</v>
       </c>
       <c r="C47" s="8" t="s">
@@ -4048,7 +4775,7 @@
       <c r="F47" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G47" s="16"/>
+      <c r="G47" s="14"/>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
       <c r="J47" s="8"/>
@@ -4099,10 +4826,10 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="7">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
@@ -4117,10 +4844,10 @@
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="7">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
@@ -4135,10 +4862,10 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="7">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
@@ -4151,264 +4878,680 @@
       <c r="I52" s="9"/>
       <c r="J52" s="9"/>
     </row>
-    <row r="53" spans="1:10" ht="20.25">
-      <c r="A53" s="40" t="s">
+    <row r="53" spans="1:10" ht="33">
+      <c r="A53" s="7">
+        <v>50</v>
+      </c>
+      <c r="B53" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="D53" s="38"/>
+      <c r="E53" s="38"/>
+      <c r="F53" s="12"/>
+      <c r="G53" s="38"/>
+      <c r="H53" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I53" s="9"/>
+      <c r="J53" s="9" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="16.5">
+      <c r="A54" s="7">
+        <v>51</v>
+      </c>
+      <c r="B54" s="39" t="s">
+        <v>191</v>
+      </c>
+      <c r="C54" s="38" t="s">
+        <v>192</v>
+      </c>
+      <c r="D54" s="38"/>
+      <c r="E54" s="38"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="38"/>
+      <c r="H54" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I54" s="9"/>
+      <c r="J54" s="9" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="20.25">
+      <c r="A55" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="B53" s="41"/>
-      <c r="C53" s="41"/>
-      <c r="D53" s="41"/>
-      <c r="E53" s="42"/>
-      <c r="F53" s="4">
+      <c r="B55" s="47"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="47"/>
+      <c r="E55" s="48"/>
+      <c r="F55" s="4">
         <f>COUNTA(F4:F52)</f>
         <v>6</v>
       </c>
-      <c r="G53" s="4">
+      <c r="G55" s="4">
         <f>COUNTA(G4:G52)</f>
         <v>0</v>
       </c>
-      <c r="H53" s="4">
-        <f>COUNTA(H4:H52)</f>
-        <v>4</v>
-      </c>
-      <c r="I53" s="4">
+      <c r="H55" s="4">
+        <f>COUNTA(H4:H54)</f>
+        <v>6</v>
+      </c>
+      <c r="I55" s="4">
         <f>COUNTA(I4:I52)</f>
         <v>39</v>
       </c>
-      <c r="J53" s="9"/>
-    </row>
-    <row r="54" spans="1:10" ht="20.25">
-      <c r="A54" s="17"/>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="18"/>
-      <c r="H54" s="18"/>
-      <c r="I54" s="18"/>
-    </row>
-    <row r="55" spans="1:10" ht="20.25">
-      <c r="A55" s="17"/>
-      <c r="B55" s="17" t="s">
+      <c r="J55" s="9"/>
+    </row>
+    <row r="56" spans="1:10" ht="20.25">
+      <c r="A56" s="15"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
+      <c r="H56" s="49">
+        <f>H55+I55</f>
+        <v>45</v>
+      </c>
+      <c r="I56" s="49"/>
+    </row>
+    <row r="57" spans="1:10" ht="20.25">
+      <c r="A57" s="15"/>
+      <c r="B57" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C57" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="18"/>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="18"/>
-    </row>
-    <row r="56" spans="1:10">
-      <c r="B56" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10">
-      <c r="B57" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
-      <c r="B58" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10">
-      <c r="B59" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
-      <c r="B60" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="28.5">
-      <c r="B61" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10">
-      <c r="B62" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10">
-      <c r="B63" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="15" thickBot="1">
-      <c r="B64" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" ht="15" thickBot="1">
-      <c r="B65" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="66" spans="2:5">
-      <c r="B66" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="67" spans="2:5">
-      <c r="B67" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="2:5">
-      <c r="B68" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D68" s="15"/>
-      <c r="E68" s="15"/>
-    </row>
-    <row r="69" spans="2:5">
-      <c r="B69" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>50</v>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
+    </row>
+    <row r="58" spans="1:10" ht="36.75" customHeight="1">
+      <c r="A58" s="40">
+        <v>1</v>
+      </c>
+      <c r="B58" s="62" t="s">
+        <v>193</v>
+      </c>
+      <c r="C58" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E58" s="15"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
+    </row>
+    <row r="59" spans="1:10" ht="40.5" customHeight="1">
+      <c r="A59" s="40">
+        <v>2</v>
+      </c>
+      <c r="B59" s="62" t="s">
+        <v>195</v>
+      </c>
+      <c r="C59" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
+    </row>
+    <row r="60" spans="1:10" ht="52.5" customHeight="1">
+      <c r="A60" s="40">
+        <v>3</v>
+      </c>
+      <c r="B60" s="62" t="s">
+        <v>196</v>
+      </c>
+      <c r="C60" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E60" s="15"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="16"/>
+      <c r="I60" s="16"/>
+    </row>
+    <row r="61" spans="1:10" ht="53.25" customHeight="1">
+      <c r="A61" s="40">
+        <v>4</v>
+      </c>
+      <c r="B61" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="C61" s="42" t="s">
+        <v>198</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E61" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="16"/>
+      <c r="I61" s="16"/>
+    </row>
+    <row r="62" spans="1:10" ht="51" customHeight="1">
+      <c r="A62" s="40">
+        <v>5</v>
+      </c>
+      <c r="B62" s="41" t="s">
+        <v>199</v>
+      </c>
+      <c r="C62" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D62" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E62" s="65" t="s">
+        <v>214</v>
+      </c>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="16"/>
+      <c r="I62" s="16"/>
+    </row>
+    <row r="63" spans="1:10" ht="42" customHeight="1">
+      <c r="A63" s="40">
+        <v>6</v>
+      </c>
+      <c r="B63" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="C63" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E63" s="66"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16"/>
+    </row>
+    <row r="64" spans="1:10" ht="42" customHeight="1">
+      <c r="A64" s="40">
+        <v>7</v>
+      </c>
+      <c r="B64" s="41" t="s">
+        <v>201</v>
+      </c>
+      <c r="C64" s="61" t="s">
+        <v>194</v>
+      </c>
+      <c r="D64" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E64" s="66" t="s">
+        <v>214</v>
+      </c>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
+    </row>
+    <row r="65" spans="1:9" ht="42" customHeight="1">
+      <c r="A65" s="40">
+        <v>8</v>
+      </c>
+      <c r="B65" s="41" t="s">
+        <v>202</v>
+      </c>
+      <c r="C65" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D65" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E65" s="66" t="s">
+        <v>214</v>
+      </c>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="16"/>
+    </row>
+    <row r="66" spans="1:9" ht="42" customHeight="1">
+      <c r="A66" s="40">
+        <v>9</v>
+      </c>
+      <c r="B66" s="43" t="s">
+        <v>203</v>
+      </c>
+      <c r="C66" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D66" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E66" s="66" t="s">
+        <v>214</v>
+      </c>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16"/>
+      <c r="H66" s="16"/>
+      <c r="I66" s="16"/>
+    </row>
+    <row r="67" spans="1:9" ht="42" customHeight="1">
+      <c r="A67" s="40">
+        <v>10</v>
+      </c>
+      <c r="B67" s="43" t="s">
+        <v>204</v>
+      </c>
+      <c r="C67" s="42"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="66"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="16"/>
+      <c r="I67" s="16"/>
+    </row>
+    <row r="68" spans="1:9" ht="42" customHeight="1">
+      <c r="A68" s="40">
+        <v>12</v>
+      </c>
+      <c r="B68" s="43" t="s">
+        <v>205</v>
+      </c>
+      <c r="C68" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E68" s="66" t="s">
+        <v>214</v>
+      </c>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="16"/>
+    </row>
+    <row r="69" spans="1:9" ht="42" customHeight="1">
+      <c r="A69" s="40">
+        <v>13</v>
+      </c>
+      <c r="B69" s="64" t="s">
+        <v>206</v>
+      </c>
+      <c r="C69" s="63" t="s">
+        <v>194</v>
       </c>
       <c r="D69" s="15"/>
       <c r="E69" s="15"/>
-    </row>
-    <row r="70" spans="2:5" ht="28.5">
-      <c r="B70" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>50</v>
-      </c>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="16"/>
+    </row>
+    <row r="70" spans="1:9" ht="54" customHeight="1">
+      <c r="A70" s="40">
+        <v>15</v>
+      </c>
+      <c r="B70" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="C70" s="42"/>
       <c r="D70" s="15"/>
       <c r="E70" s="15"/>
-    </row>
-    <row r="71" spans="2:5" ht="28.5">
-      <c r="B71" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>50</v>
-      </c>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="16"/>
+      <c r="I70" s="16"/>
+    </row>
+    <row r="71" spans="1:9" ht="42" customHeight="1">
+      <c r="A71" s="40">
+        <v>16</v>
+      </c>
+      <c r="B71" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="C71" s="42"/>
       <c r="D71" s="15"/>
       <c r="E71" s="15"/>
-    </row>
-    <row r="72" spans="2:5">
-      <c r="B72" s="15" t="s">
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
+      <c r="H71" s="16"/>
+      <c r="I71" s="16"/>
+    </row>
+    <row r="72" spans="1:9" ht="42" customHeight="1">
+      <c r="A72" s="40">
+        <v>17</v>
+      </c>
+      <c r="B72" s="43" t="s">
+        <v>209</v>
+      </c>
+      <c r="C72" s="42"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="16"/>
+      <c r="G72" s="16"/>
+      <c r="H72" s="16"/>
+      <c r="I72" s="16"/>
+    </row>
+    <row r="73" spans="1:9" ht="20.25">
+      <c r="A73" s="40">
+        <v>18</v>
+      </c>
+      <c r="B73" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="C73" s="42"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
+      <c r="F73" s="16"/>
+      <c r="G73" s="16"/>
+      <c r="H73" s="16"/>
+      <c r="I73" s="16"/>
+    </row>
+    <row r="74" spans="1:9" ht="20.25">
+      <c r="A74" s="15"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="15"/>
+      <c r="F74" s="16"/>
+      <c r="G74" s="16"/>
+      <c r="H74" s="16"/>
+      <c r="I74" s="16"/>
+    </row>
+    <row r="75" spans="1:9" ht="20.25">
+      <c r="A75" s="15"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="15"/>
+      <c r="D75" s="15"/>
+      <c r="E75" s="15"/>
+      <c r="F75" s="16"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="16"/>
+      <c r="I75" s="16"/>
+    </row>
+    <row r="76" spans="1:9" ht="20.25">
+      <c r="A76" s="15"/>
+      <c r="B76" s="15"/>
+      <c r="C76" s="15"/>
+      <c r="D76" s="15"/>
+      <c r="E76" s="15"/>
+      <c r="F76" s="16"/>
+      <c r="G76" s="16"/>
+      <c r="H76" s="16"/>
+      <c r="I76" s="16"/>
+    </row>
+    <row r="77" spans="1:9" ht="20.25">
+      <c r="A77" s="15"/>
+      <c r="B77" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15"/>
+      <c r="F77" s="16"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="16"/>
+      <c r="I77" s="16"/>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" s="17">
+        <v>1</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" s="17">
+        <v>2</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" s="17">
+        <v>3</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="17">
+        <v>4</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="17">
+        <v>5</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="15" thickBot="1">
+      <c r="A83" s="17">
+        <v>6</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="15" thickBot="1">
+      <c r="A84" s="17">
+        <v>7</v>
+      </c>
+      <c r="B84" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="17">
+        <v>8</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="17">
+        <v>9</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D86" s="13"/>
+      <c r="E86" s="13"/>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="17">
+        <v>10</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D87" s="13"/>
+      <c r="E87" s="13"/>
+    </row>
+    <row r="88" spans="1:5" ht="28.5">
+      <c r="A88" s="17">
+        <v>11</v>
+      </c>
+      <c r="B88" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D88" s="13"/>
+      <c r="E88" s="13"/>
+    </row>
+    <row r="89" spans="1:5" ht="28.5">
+      <c r="A89" s="17">
+        <v>12</v>
+      </c>
+      <c r="B89" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D89" s="13"/>
+      <c r="E89" s="13"/>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" s="17">
+        <v>13</v>
+      </c>
+      <c r="B90" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C90" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" s="17">
+        <v>14</v>
+      </c>
+      <c r="B91" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92" s="17">
+        <v>15</v>
+      </c>
+      <c r="B92" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C92" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93" s="17">
+        <v>16</v>
+      </c>
+      <c r="B93" s="13" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="73" spans="2:5">
-      <c r="B73" s="15" t="s">
+      <c r="C93" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94" s="17">
+        <v>17</v>
+      </c>
+      <c r="B94" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C73" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="74" spans="2:5">
-      <c r="B74" s="15" t="s">
+      <c r="C94" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95" s="17">
+        <v>18</v>
+      </c>
+      <c r="B95" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C74" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="75" spans="2:5">
-      <c r="B75" s="15" t="s">
+      <c r="C95" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96" s="17">
+        <v>19</v>
+      </c>
+      <c r="B96" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C75" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="76" spans="2:5">
-      <c r="B76" s="3" t="s">
+      <c r="C96" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="17">
+        <v>20</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C76" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="77" spans="2:5">
-      <c r="B77" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C77" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="78" spans="2:5">
-      <c r="B78" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C78" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="79" spans="2:5">
-      <c r="B79" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C79" s="15" t="s">
-        <v>141</v>
+      <c r="C97" s="13" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A27:J30">
     <sortCondition ref="H27:H30"/>
   </sortState>
-  <mergeCells count="11">
-    <mergeCell ref="A53:E53"/>
+  <mergeCells count="12">
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="H56:I56"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="A2:A3"/>
@@ -4418,7 +5561,7 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="J43:J45"/>
+    <mergeCell ref="J43:J44"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4431,59 +5574,59 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9" style="25"/>
-    <col min="2" max="2" width="17.875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="52.375" style="31" customWidth="1"/>
-    <col min="4" max="4" width="97.125" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.125" style="25" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="25"/>
+    <col min="1" max="1" width="9" style="22"/>
+    <col min="2" max="2" width="17.875" style="22" customWidth="1"/>
+    <col min="3" max="3" width="52.375" style="28" customWidth="1"/>
+    <col min="4" max="4" width="97.125" style="22" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.125" style="22" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="22"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
-      <c r="C1" s="24"/>
+      <c r="C1" s="21"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:5" ht="38.25">
-      <c r="A2" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="B2" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="C2" s="35" t="s">
+      <c r="A2" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="D2" s="35" t="s">
-        <v>168</v>
-      </c>
-      <c r="E2" s="35" t="s">
-        <v>170</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="50" t="s">
-        <v>164</v>
-      </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="52"/>
+      <c r="A3" s="58" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="60"/>
     </row>
     <row r="4" spans="1:5" ht="29.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>157</v>
+        <v>148</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>154</v>
       </c>
       <c r="E4" s="1"/>
     </row>
@@ -4492,79 +5635,79 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="60">
+      <c r="A6" s="29">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" ht="29.25">
+      <c r="A7" s="29">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C5" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" s="28" t="s">
+      <c r="C7" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" ht="60">
-      <c r="A6" s="32">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="28" t="s">
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" ht="68.25" customHeight="1">
+      <c r="A8" s="29">
+        <v>5</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" ht="29.25">
-      <c r="A7" s="32">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="C7" s="28" t="s">
+      <c r="D8" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="D7" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" ht="68.25" customHeight="1">
-      <c r="A8" s="32">
-        <v>5</v>
-      </c>
-      <c r="B8" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>163</v>
-      </c>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="52"/>
+      <c r="A9" s="58" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="60"/>
     </row>
     <row r="10" spans="1:5" ht="29.25">
       <c r="A10" s="1">
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>165</v>
+        <v>148</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>162</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -4572,142 +5715,142 @@
     <row r="11" spans="1:5">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
-      <c r="C11" s="27"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="27"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="27"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="27"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="27"/>
+      <c r="C15" s="24"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
-      <c r="C16" s="27"/>
+      <c r="C16" s="24"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
-      <c r="C17" s="27"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="27"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="27"/>
+      <c r="C19" s="24"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
-      <c r="C20" s="27"/>
+      <c r="C20" s="24"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
-      <c r="C21" s="27"/>
+      <c r="C21" s="24"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="27"/>
+      <c r="C22" s="24"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
-      <c r="C23" s="27"/>
+      <c r="C23" s="24"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
-      <c r="C24" s="27"/>
+      <c r="C24" s="24"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
-      <c r="C25" s="27"/>
+      <c r="C25" s="24"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="A27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
+      <c r="A30" s="26"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>